<commit_message>
Correct Goodyear ACE assignment
</commit_message>
<xml_diff>
--- a/source-data/Strategic_End_User_Facilities_Bottler_Expansion_v2.xlsx
+++ b/source-data/Strategic_End_User_Facilities_Bottler_Expansion_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josephnovotny/Documents/Codex/2026-08-10/continue-my-strategic-facility-locations-map-2/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E71029-25E2-E545-A52A-062A2E9E6C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A341C086-26E4-DD4B-AC93-3F78D5800768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Facilities v2" sheetId="1" r:id="rId1"/>
@@ -3912,7 +3912,7 @@
   <autoFilter ref="A1:P258" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="7">
       <filters>
-        <filter val="ID"/>
+        <filter val="AZ"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -4467,7 +4467,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="30" hidden="1">
+    <row r="7" spans="1:16" ht="30">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -5049,7 +5049,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="30" hidden="1">
+    <row r="20" spans="1:16" ht="30">
       <c r="A20" s="2" t="s">
         <v>52</v>
       </c>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="P51" s="2"/>
     </row>
-    <row r="52" spans="1:16" ht="30" hidden="1">
+    <row r="52" spans="1:16" ht="30">
       <c r="A52" s="2" t="s">
         <v>165</v>
       </c>
@@ -6533,7 +6533,7 @@
       </c>
       <c r="P52" s="2"/>
     </row>
-    <row r="53" spans="1:16" ht="30" hidden="1">
+    <row r="53" spans="1:16" ht="30">
       <c r="A53" s="2" t="s">
         <v>165</v>
       </c>
@@ -9739,7 +9739,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="123" spans="1:16" ht="30" hidden="1">
+    <row r="123" spans="1:16" ht="30">
       <c r="A123" s="2" t="s">
         <v>364</v>
       </c>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="P140" s="2"/>
     </row>
-    <row r="141" spans="1:16" ht="15" hidden="1">
+    <row r="141" spans="1:16" ht="15">
       <c r="A141" s="2" t="s">
         <v>425</v>
       </c>
@@ -10625,7 +10625,7 @@
         <v>-112.37537741849501</v>
       </c>
       <c r="M141" s="2" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="N141" s="2" t="s">
         <v>25</v>
@@ -13995,7 +13995,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="212" spans="1:16" ht="30" hidden="1">
+    <row r="212" spans="1:16" ht="30">
       <c r="A212" s="2" t="s">
         <v>16</v>
       </c>
@@ -14195,7 +14195,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="216" spans="1:16" ht="30">
+    <row r="216" spans="1:16" ht="30" hidden="1">
       <c r="A216" s="2" t="s">
         <v>16</v>
       </c>

</xml_diff>